<commit_message>
field renaming, additional null checks and file validation
</commit_message>
<xml_diff>
--- a/src/test/resources/testfiles/importer/excel-file-importer-spec.xlsx
+++ b/src/test/resources/testfiles/importer/excel-file-importer-spec.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="string" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t xml:space="preserve">String</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t xml:space="preserve">String ends with space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">苹果</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special characters</t>
   </si>
   <si>
     <t xml:space="preserve">Numeric</t>
@@ -91,13 +97,14 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="166" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -118,6 +125,12 @@
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Noto Sans CJK SC"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -172,15 +185,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -201,8 +214,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.58"/>
   </cols>
@@ -253,6 +266,14 @@
       </c>
       <c r="B6" s="0" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -272,7 +293,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="11.5234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.25"/>
@@ -280,7 +301,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -291,7 +312,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -299,15 +320,15 @@
         <v>1.2</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -315,7 +336,7 @@
         <v>36526</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -335,14 +356,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.5234375" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.97"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -354,7 +375,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -363,7 +384,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>